<commit_message>
[FEAT] 102001 연출 완료
</commit_message>
<xml_diff>
--- a/NineReincarnation/Assets/08. Scripts/03. Data/DialogueData.xlsx
+++ b/NineReincarnation/Assets/08. Scripts/03. Data/DialogueData.xlsx
@@ -1406,7 +1406,7 @@
     <xdr:ext cx="3524250" cy="695325"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="이미지"/>
+        <xdr:cNvPr id="0" name="image2.png" title="이미지"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1434,7 +1434,7 @@
     <xdr:ext cx="1847850" cy="838200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="이미지"/>
+        <xdr:cNvPr id="0" name="image1.png" title="이미지"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1462,7 +1462,7 @@
     <xdr:ext cx="1847850" cy="838200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="이미지"/>
+        <xdr:cNvPr id="0" name="image3.png" title="이미지"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -4465,8 +4465,8 @@
         <v>Bubble</v>
       </c>
       <c r="C128" s="34">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.5)</f>
+        <v>1.5</v>
       </c>
       <c r="D128" s="34">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),201042.0)</f>
@@ -11365,10 +11365,7 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),201040.0)</f>
         <v>201040</v>
       </c>
-      <c r="B38" s="34" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Yeonong")</f>
-        <v>Yeonong</v>
-      </c>
+      <c r="B38" s="34"/>
       <c r="C38" s="34" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"ZoomIn")</f>
         <v>ZoomIn</v>
@@ -11754,8 +11751,8 @@
         <v>Yeon_wheel</v>
       </c>
       <c r="D20" s="34" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Right")</f>
-        <v>Right</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Left")</f>
+        <v>Left</v>
       </c>
     </row>
     <row r="21">
@@ -11772,8 +11769,8 @@
         <v>Yeon_wheel</v>
       </c>
       <c r="D21" s="34" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Right")</f>
-        <v>Right</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Left")</f>
+        <v>Left</v>
       </c>
     </row>
     <row r="22">
@@ -12262,8 +12259,14 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"무엇을 물을까?")</f>
         <v>무엇을 물을까?</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
+      <c r="C4" s="34" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Anna")</f>
+        <v>Anna</v>
+      </c>
+      <c r="D4" s="34">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -15055,7 +15058,7 @@
       <c r="D100" s="6">
         <v>0.0</v>
       </c>
-      <c r="E100" s="6">
+      <c r="E100" s="72">
         <v>201016.0</v>
       </c>
       <c r="F100" s="6" t="s">
@@ -15096,6 +15099,12 @@
       <c r="K101" s="60">
         <v>0.8</v>
       </c>
+      <c r="Q101" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="R101" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="72">
@@ -15317,7 +15326,7 @@
         <v>239</v>
       </c>
       <c r="N109" s="55" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="110">
@@ -15352,7 +15361,7 @@
         <v>239</v>
       </c>
       <c r="N110" s="55" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="111">
@@ -15798,9 +15807,7 @@
       </c>
       <c r="F127" s="32"/>
       <c r="G127" s="32"/>
-      <c r="H127" s="6" t="s">
-        <v>238</v>
-      </c>
+      <c r="H127" s="6"/>
       <c r="I127" s="60" t="s">
         <v>112</v>
       </c>
@@ -15828,7 +15835,7 @@
         <v>55</v>
       </c>
       <c r="D128" s="6">
-        <v>0.0</v>
+        <v>1.5</v>
       </c>
       <c r="E128" s="6">
         <v>201042.0</v>

</xml_diff>